<commit_message>
Fix Pobeda 16 name
</commit_message>
<xml_diff>
--- a/igracki.xlsx
+++ b/igracki.xlsx
@@ -3175,7 +3175,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="20.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16376" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16376" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3242,15 +3242,15 @@
       <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="0"/>
-      <c r="W1" s="0"/>
-      <c r="X1" s="0"/>
-      <c r="Y1" s="0"/>
-      <c r="Z1" s="0"/>
-      <c r="AA1" s="0"/>
-      <c r="AB1" s="0"/>
-      <c r="AC1" s="0"/>
-      <c r="AD1" s="0"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -4256,7 +4256,7 @@
         <v>35858</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="I38" s="1" t="n">
         <v>20</v>

</xml_diff>